<commit_message>
chore(ejemplos): regenerar licitación de ejemplo
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ejemplos/licitacion_ejemplo.xlsx
+++ b/ejemplos/licitacion_ejemplo.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TEE HD EXTREMO JUNTA HIDRÁULICA 12"X 12" (SUMINISTRO E INSTALACIÓN)</t>
+          <t>CONSTRUCCIÓN INTERSECCIÓN A DESNIVEL PUENTE ARANDA Y DEMÁS OBRAS COMPLEMENTARIAS TRONCAL CALLE 13 - VÁLVULA COMPUERTA VNA Ø2" HD B16.5 CL 300 CON VOLANTE MANIOBRA.  (Incluye suministro e instalación)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>203.05</v>
+        <v>332.2</v>
       </c>
       <c r="E2" t="n">
-        <v>5461640</v>
+        <v>1226458</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -484,19 +484,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MEZCLA ASFÁLTICA EN CALIENTE TIPO DENSO MD10 ASFALTO 80-100 (INCLUYE SUMINISTRO, EXTENDIDO, NIVELACIÓN, COMPACTACIÓN MECANICA CON VIBROCOMPACTADOR Y COMPACTADOR DE LLANTAS, FACTOR DE COMPACTACION Y TRANSPORTE DE MATERIAL A 21 KMS)</t>
+          <t>BASE EN CONCRETO 3000 PSI HECHO EN OBRA PARA POSTE METÁLICO H=14M (INCLUYE SUMINISTRO Y CONSTRUCCIÓN. INCLUYE REFUERZO) NORMA AP802.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>UN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>156.83</v>
+        <v>360.84</v>
       </c>
       <c r="E3" t="n">
-        <v>1268217</v>
+        <v>567808</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -512,19 +512,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Suministro e instalación de 2 ductos d=3" pvc-eb (incluye suministro e instalación. no incluye rellenos). cs207.</t>
+          <t>Obra de bolardo en hierro tipo m63 (suministro e instalación. incluye base en concreto 1500 psi, hecho obra)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>UN</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>51.4</v>
+        <v>200.86</v>
       </c>
       <c r="E4" t="n">
-        <v>50218</v>
+        <v>329461</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CODO 90° CXE PVC SANITARIA D=6" (INCLUYE SUMINISTRO E INSTALACIÓN).</t>
+          <t>FALSO PIMIENTO H=1.3M (INCLUYE SIEMBRA, TIERRA, ABONO Y TUTOR) INCLUYE TRANSPORTE Y DISPOSICIÓN FINAL DE ESCOMBROS EN SITIO AUTORIZADO A 28 KM). SUMINISTRO Y PLANTACION.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -549,10 +549,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>479.24</v>
+        <v>169.81</v>
       </c>
       <c r="E5" t="n">
-        <v>202630</v>
+        <v>257041</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -568,19 +568,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MEZCLA ASFÁLTICA DENSA EN CALIENTE MD12 CON CEMENTO ASFÁLTICO 60-70 (SUMINISTRO, EXTENDIDO, NIVELACIÓN Y COMPACTACIÓN MECANICA CON VIBROCOMPACTADOR Y COMPACTADOR DE LLANTAS)</t>
+          <t>KIT DE NIVELACIÓN PARA HIDRANTE DE DIÁMETRO DE 6", LONGITUD 400MM. SUMINISTRO E INSTALACIÓN. (INCLUYE TRANSPORTE Y TODOS LOS ELEMENTOS NECESARIOS PARA SU INSTALACIÓN).</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>UN</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>428.09</v>
+        <v>492.52</v>
       </c>
       <c r="E6" t="n">
-        <v>1038692</v>
+        <v>1688332</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Obra de construcción de la intersección a de puente aranda - concreto 4000 psi grava común ( 28 mpa) para estribos (premezclado. incluye suministro, formaleteo, bombeo, colocación y curado. no incluye refuerzo)</t>
+          <t>Ejecución de construcción de la intersección a de puente aranda - concreto 4000 psi grava común ( 28 mpa) para estribos (premezclado. incluye suministro, formaleteo, bombeo, colocación y curado. no incluye refuerzo)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>447.47</v>
+        <v>364.84</v>
       </c>
       <c r="E7" t="n">
         <v>1104872</v>
@@ -624,19 +624,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXCAVACION MECANICA PARA REDES PROFUNDIDAD MAYORES A 3.5M (INCLUYE CARGUE).</t>
+          <t>2 DUCTOS D=3" PVC-EB (INCLUYE SUMINISTRO E INSTALACIÓN. NO INCLUYE RELLENOS). NORMA CS207.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>394.18</v>
+        <v>325.18</v>
       </c>
       <c r="E8" t="n">
-        <v>6921</v>
+        <v>50218</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -652,19 +652,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RELLENO EN TRITURADO DE 3/4`` (INCLUYE TRANSPORTE, SUMINISTRO, EXTENDIDO MANUAL Y COLOCACIÓN)</t>
+          <t>2 DUCTOS D=2" PVC PESADO DB. SUMINISTRO E INSTALACION. (NO INCLUYE RELLENOS).</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>302.31</v>
+        <v>31.46</v>
       </c>
       <c r="E9" t="n">
-        <v>184517</v>
+        <v>16879</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ejecución de construcción intersección a desnivel puente aranda y demás obras complementarias troncal calle 13 - válvula tipo mariposa de ø 36", astm a536, cl 300 #, extremos bridados ansi/asme b16.47 (suministro e instalación)</t>
+          <t>Obra de plantacion de palma alejandra h= 1.5 m. (incluye suministro al sitio de obra, plantacion, aplicación y mezcla de sustrato, tutor y amarre. incluye transporte y disposición final de en sitio autorizadoa 28 km).</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>363.13</v>
+        <v>353.52</v>
       </c>
       <c r="E10" t="n">
-        <v>59583475</v>
+        <v>365093</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -708,19 +708,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IMPERMEABILIZANTE PARA CONCRETO. SUMINISTRO Y APLICACIÓN</t>
+          <t>PARADERO TIPO M10 (INC. SUM. E INST. INC. BASES EN CONCRETO 3000 PSI, HECHO EN OBRA. NO INCLUYE LOSAS DE CONCRETO)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>UN</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>252.15</v>
+        <v>257.72</v>
       </c>
       <c r="E11" t="n">
-        <v>3652</v>
+        <v>13813639</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAJA DE MANIOBRA ENTRADA Y SALIDA SUBESTACION SEMISUMERGIBLE NORMA CODENSA CTS535. SUMINISTRO E INSTALACION.</t>
+          <t>DESMONTE DE PARADERO URBANO TIPO M10 (INCLUYE CARGUE Y TRANSPORTE A ALMACEN AUTORIZADO POR EL IDU.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>149.25</v>
+        <v>455.84</v>
       </c>
       <c r="E12" t="n">
-        <v>19008635</v>
+        <v>640737</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -764,19 +764,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Obra de pisos en loseta prefabricada a55 táctil alerta o a56 guia 40x40x6 cm. suministro e instalación. (incluye 4cm de mortero 1:5 en obra para base y arena de peña para sello).</t>
+          <t>Obra de valla transversal de señalizacion para acceso a estacion (335x32cm) en vinilo adhesivo sobre alucobond de 4mm. segun cartilla de señaletica transmilenio 2023 para estaciones tipo ancho 5 mt. (incluye suministro e instalación)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>UN</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>80.93000000000001</v>
+        <v>288.55</v>
       </c>
       <c r="E13" t="n">
-        <v>140275</v>
+        <v>4501426</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -801,10 +801,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>66.86</v>
+        <v>65.97</v>
       </c>
       <c r="E14" t="n">
-        <v>300254</v>
+        <v>55628</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>43.47</v>
+        <v>56.49</v>
       </c>
       <c r="E15" t="n">
-        <v>200236</v>
+        <v>329289</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -857,10 +857,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>57.58</v>
+        <v>58.34</v>
       </c>
       <c r="E16" t="n">
-        <v>226939</v>
+        <v>384627</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>

</xml_diff>